<commit_message>
going back to multiple data sources
</commit_message>
<xml_diff>
--- a/input/Template_EMIS_Access_PTR_protection.xlsx
+++ b/input/Template_EMIS_Access_PTR_protection.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="469" documentId="8_{D63770E9-8D5C-4F2A-BD7D-98D3C6683B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B793117-7AB4-49DD-B3A2-3AEDF5B7A79E}"/>
   <bookViews>
-    <workbookView xWindow="28905" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{24D09A16-471A-4A7F-BD10-C475AB78837D}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="1870" windowWidth="5105" windowHeight="3290" xr2:uid="{24D09A16-471A-4A7F-BD10-C475AB78837D}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator" sheetId="3" r:id="rId1"/>

</xml_diff>